<commit_message>
Remove ai_sdd entirely (SDD generation skill)
</commit_message>
<xml_diff>
--- a/work/tst_mdl/Foc_2024b_signals_cal.xlsx
+++ b/work/tst_mdl/Foc_2024b_signals_cal.xlsx
@@ -7,13 +7,14 @@
   </bookViews>
   <sheets>
     <sheet name="Signals" sheetId="1" r:id="rId2"/>
+    <sheet name="Calibration" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="444" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="729" uniqueCount="127">
   <si>
     <t>PortName</t>
   </si>
@@ -316,6 +317,84 @@
   </si>
   <si>
     <t>Foc_2024b/u16SvmDutyW</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>cal_AdcMaxCountsHw</t>
+  </si>
+  <si>
+    <t>cal_AdcRefVoltHw</t>
+  </si>
+  <si>
+    <t>cal_OhmRShuntHw</t>
+  </si>
+  <si>
+    <t>cal_GainAmpHw</t>
+  </si>
+  <si>
+    <t>cal_AdcVoltMidHw</t>
+  </si>
+  <si>
+    <t>cal_FullScaleCur</t>
+  </si>
+  <si>
+    <t>cal_u8TiDebPhaCur</t>
+  </si>
+  <si>
+    <t>cal_s16ThresholdPhaCurImplaisible</t>
+  </si>
+  <si>
+    <t>cal_s16Inductivity</t>
+  </si>
+  <si>
+    <t>cal_s16RPha</t>
+  </si>
+  <si>
+    <t>cal_s16LpfPllEst</t>
+  </si>
+  <si>
+    <t>cal_s16LpfPllEstOpenLoop</t>
+  </si>
+  <si>
+    <t>cal_s16OmegaGainEst</t>
+  </si>
+  <si>
+    <t>cal_HwtDutyU</t>
+  </si>
+  <si>
+    <t>cal_HwtDutyV</t>
+  </si>
+  <si>
+    <t>cal_HwtDutyW</t>
+  </si>
+  <si>
+    <t>cal_HwtSector</t>
+  </si>
+  <si>
+    <t>cal_bActHwMode</t>
+  </si>
+  <si>
+    <t>cal_s16MinSampleTime</t>
+  </si>
+  <si>
+    <t>BlockType</t>
+  </si>
+  <si>
+    <t>Constant</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Unit</t>
   </si>
 </sst>
 </file>
@@ -1260,4 +1339,368 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="32.42578125" customWidth="true"/>
+    <col min="2" max="2" width="10.140625" customWidth="true"/>
+    <col min="3" max="3" width="12.140625" customWidth="true"/>
+    <col min="4" max="4" width="32.42578125" customWidth="true"/>
+    <col min="5" max="5" width="4.5703125" customWidth="true"/>
+    <col min="6" max="6" width="4.85546875" customWidth="true"/>
+    <col min="7" max="7" width="4.85546875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="E8" s="0"/>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" s="0"/>
+      <c r="F9" s="0"/>
+      <c r="G9" s="0"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="0"/>
+      <c r="F10" s="0"/>
+      <c r="G10" s="0"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" s="0"/>
+      <c r="F11" s="0"/>
+      <c r="G11" s="0"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="E12" s="0"/>
+      <c r="F12" s="0"/>
+      <c r="G12" s="0"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="E13" s="0"/>
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="E14" s="0"/>
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="E15" s="0"/>
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="E17" s="0"/>
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="E19" s="0"/>
+      <c r="F19" s="0"/>
+      <c r="G19" s="0"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="E20" s="0"/>
+      <c r="F20" s="0"/>
+      <c r="G20" s="0"/>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>